<commit_message>
Session 23: UX feedback, cost model, whitepaper v3, 5-wave launch emails
- FEA: Featured carousel desktop arrows, photo lightbox, My Requests tab,
  back buttons (Browse/Saved/Wallet/Recruit), placeholder sort fix,
  credentials string/object fix, Trust Score composition note
- Cost model: ZAR/USD rate, accountant R2k, software R500, SA tax 27%,
  Revenue vs Cost unit format fix
- TrustSquare_WhitePaper_v3.docx: 7 patent claims, dual-entity IP structure,
  5 timestamp authorities, trademark + provisional patent filing guide
- TrustSquare_LaunchEmails_5Wave.docx: 5-wave campaign for Pretoria agents,
  KW RSA, and global outreach
</commit_message>
<xml_diff>
--- a/Cost_Breakdown_GlobalLaunch.xlsx
+++ b/Cost_Breakdown_GlobalLaunch.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Assumptions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Wave Growth" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Operating Costs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Revenue vs Cost" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Dashboard" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wave Growth" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operating Costs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue vs Cost" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -19,10 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="$#,##0"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -116,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -134,6 +135,7 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -393,7 +395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C74"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1040,153 +1042,168 @@
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="15" t="inlineStr">
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ZAR / USD exchange rate</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>R18.50 per $1 — used to convert ZAR costs to USD (update periodically)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="15" t="inlineStr">
         <is>
           <t>AI COACH — ADVERT AGENT</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>AI Coach adoption rate (% of active sellers)</t>
-        </is>
-      </c>
-      <c r="B64" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>15% of active sellers purchase &gt;= 1 pack per year</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Avg packs per adopting seller per year</t>
+          <t>AI Coach adoption rate (% of active sellers)</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>2</v>
+        <v>0.15</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>T spent per adopting seller per year across all tiers</t>
+          <t>15% of active sellers purchase &gt;= 1 pack per year</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
+          <t>Avg packs per adopting seller per year</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>2</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>T spent per adopting seller per year across all tiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
           <t>Anthropic API cost per session (USD)</t>
         </is>
       </c>
-      <c r="B66" t="n">
+      <c r="B67" t="n">
         <v>0.01</v>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C67" t="inlineStr">
         <is>
           <t>Haiku 4.5 — est. 800 in + 400 out tokens per session</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="15" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="15" t="inlineStr">
         <is>
           <t>TIERED AI PACK PRICING</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Tier 1 — 5T · 40 AI uses</t>
-        </is>
-      </c>
-      <c r="B69" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Entry tier · 8 uses per Tuppence</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Tier 2 — 10T · 100 AI uses</t>
+          <t>Tier 1 — 5T · 40 AI uses</t>
         </is>
       </c>
       <c r="B70" s="16" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Standard tier · 10 uses per Tuppence</t>
+          <t>Entry tier · 8 uses per Tuppence</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Tier 3 — 25T · 320 AI uses</t>
+          <t>Tier 2 — 10T · 100 AI uses</t>
         </is>
       </c>
       <c r="B71" s="16" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Best value · 12.8 uses per Tuppence</t>
+          <t>Standard tier · 10 uses per Tuppence</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Sessions per T — Tier 1</t>
-        </is>
-      </c>
-      <c r="B72">
-        <f>40/B69</f>
-        <v/>
+          <t>Tier 3 — 25T · 320 AI uses</t>
+        </is>
+      </c>
+      <c r="B72" s="16" t="n">
+        <v>25</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>8 sessions per Tuppence</t>
+          <t>Best value · 12.8 uses per Tuppence</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Sessions per T — Tier 2</t>
+          <t>Sessions per T — Tier 1</t>
         </is>
       </c>
       <c r="B73">
-        <f>100/B70</f>
+        <f>40/B69</f>
         <v/>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>10 sessions per Tuppence</t>
+          <t>8 sessions per Tuppence</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
+          <t>Sessions per T — Tier 2</t>
+        </is>
+      </c>
+      <c r="B74">
+        <f>100/B70</f>
+        <v/>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>10 sessions per Tuppence</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
           <t>Blended sessions per T (equal pack mix)</t>
         </is>
       </c>
-      <c r="B74">
+      <c r="B75">
         <f>(B72+B73+320/B71)/3</f>
         <v/>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>~10.27 — used in Operating Costs Anthropic formula</t>
         </is>
@@ -2455,7 +2472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2746,15 +2763,15 @@
         </is>
       </c>
       <c r="B20">
-        <f>ROUND('Wave Growth'!B32*Assumptions!B64*Assumptions!B65*Assumptions!$B$74*Assumptions!B66,0)</f>
+        <f>ROUND('Wave Growth'!B32*Assumptions!B65*Assumptions!B66*Assumptions!$B$75*Assumptions!B67,0)</f>
         <v/>
       </c>
       <c r="C20">
-        <f>ROUND('Wave Growth'!C32*Assumptions!B64*Assumptions!B65*Assumptions!$B$74*Assumptions!B66,0)</f>
+        <f>ROUND('Wave Growth'!C32*Assumptions!B65*Assumptions!B66*Assumptions!$B$75*Assumptions!B67,0)</f>
         <v/>
       </c>
       <c r="D20">
-        <f>ROUND('Wave Growth'!D32*Assumptions!B64*Assumptions!B65*Assumptions!$B$74*Assumptions!B66,0)</f>
+        <f>ROUND('Wave Growth'!D32*Assumptions!B65*Assumptions!B66*Assumptions!$B$75*Assumptions!B67,0)</f>
         <v/>
       </c>
       <c r="E20" t="inlineStr">
@@ -2864,59 +2881,128 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Accountant (R2,000/mo)</t>
+        </is>
+      </c>
+      <c r="B28" s="17">
+        <f>ROUND(2000/Assumptions!$B$62*12,0)</f>
+        <v/>
+      </c>
+      <c r="C28" s="17">
+        <f>B28</f>
+        <v/>
+      </c>
+      <c r="D28" s="17">
+        <f>B28</f>
+        <v/>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>R2,000/mo — monthly retainer, converted at Assumptions ZAR/USD rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Accountant software package (R500/mo)</t>
+        </is>
+      </c>
+      <c r="B29" s="17">
+        <f>ROUND(500/Assumptions!$B$62*12,0)</f>
+        <v/>
+      </c>
+      <c r="C29" s="17">
+        <f>B29</f>
+        <v/>
+      </c>
+      <c r="D29" s="17">
+        <f>B29</f>
+        <v/>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>R500/mo — accounting software (e.g. Xero/Sage), converted at Assumptions ZAR/USD rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   SA Corporate Tax (27% on net profit)</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>27% SA corporate tax on net profit — Year 1 pre-profit = $0. Update B30:D30 once P&amp;L is finalised.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15.6" customHeight="1">
+      <c r="A31" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Marketing / SaaS</t>
         </is>
       </c>
-      <c r="B28" s="11" t="n">
+      <c r="B31" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="C28" s="11" t="n">
+      <c r="C31" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="D28" s="11" t="n">
+      <c r="D31" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>Zero — n8n auto-scraping is the acquisition engine</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">   Subtotal: Overhead</t>
         </is>
       </c>
-      <c r="B29" s="11">
-        <f>SUM(B26:B28)</f>
-        <v/>
-      </c>
-      <c r="C29" s="11">
-        <f>SUM(C26:C28)</f>
-        <v/>
-      </c>
-      <c r="D29" s="11">
-        <f>SUM(D26:D28)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="15.6" customHeight="1">
-      <c r="A31" s="12" t="inlineStr">
+      <c r="B32" s="11">
+        <f>SUM(B26:B31)</f>
+        <v/>
+      </c>
+      <c r="C32" s="11">
+        <f>SUM(C26:C31)</f>
+        <v/>
+      </c>
+      <c r="D32" s="11">
+        <f>SUM(D26:D31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t>TOTAL OPERATING COSTS (USD)</t>
         </is>
       </c>
-      <c r="B31" s="11">
-        <f>B14+B19+B23+B29</f>
-        <v/>
-      </c>
-      <c r="C31" s="11">
-        <f>C14+C19+C23+C29</f>
-        <v/>
-      </c>
-      <c r="D31" s="11">
-        <f>D14+D19+D23+D29</f>
+      <c r="B34" s="11">
+        <f>B14+B19+B23+B32</f>
+        <v/>
+      </c>
+      <c r="C34" s="11">
+        <f>C14+C19+C23+C32</f>
+        <v/>
+      </c>
+      <c r="D34" s="11">
+        <f>D14+D19+D23+D32</f>
         <v/>
       </c>
     </row>
@@ -3022,15 +3108,15 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>ROUND('Wave Growth'!B32*Assumptions!B64*Assumptions!B65*Assumptions!B31,0)</f>
+        <f>ROUND('Wave Growth'!B32*Assumptions!B65*Assumptions!B66*Assumptions!B31,0)</f>
         <v/>
       </c>
       <c r="C8" s="11">
-        <f>ROUND('Wave Growth'!C32*Assumptions!B64*Assumptions!B65*Assumptions!B31,0)</f>
+        <f>ROUND('Wave Growth'!C32*Assumptions!B65*Assumptions!B66*Assumptions!B31,0)</f>
         <v/>
       </c>
       <c r="D8" s="11">
-        <f>ROUND('Wave Growth'!D32*Assumptions!B64*Assumptions!B65*Assumptions!B31,0)</f>
+        <f>ROUND('Wave Growth'!D32*Assumptions!B65*Assumptions!B66*Assumptions!B31,0)</f>
         <v/>
       </c>
     </row>
@@ -3124,15 +3210,15 @@
         </is>
       </c>
       <c r="B14" s="11">
-        <f>'Operating Costs'!B29</f>
+        <f>'Operating Costs'!B32</f>
         <v/>
       </c>
       <c r="C14" s="11">
-        <f>'Operating Costs'!C29</f>
+        <f>'Operating Costs'!C32</f>
         <v/>
       </c>
       <c r="D14" s="11">
-        <f>'Operating Costs'!D29</f>
+        <f>'Operating Costs'!D32</f>
         <v/>
       </c>
     </row>
@@ -3206,15 +3292,15 @@
           <t>Live cities</t>
         </is>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="10">
         <f>'Wave Growth'!B31</f>
         <v/>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="10">
         <f>'Wave Growth'!C31</f>
         <v/>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="10">
         <f>'Wave Growth'!D31</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
BEE-LADY-2: two real Tutors adverts (274 course R1200, 275 talks R50pp) + SUPER-CRED-2 seller-level LM evidence model in credentials endpoint
</commit_message>
<xml_diff>
--- a/Cost_Breakdown_GlobalLaunch.xlsx
+++ b/Cost_Breakdown_GlobalLaunch.xlsx
@@ -26,7 +26,7 @@
     <numFmt numFmtId="167" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -101,8 +101,12 @@
       <color rgb="FFFF8C00"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -139,6 +143,11 @@
         <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E75B6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -159,7 +168,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -344,6 +353,8 @@
     <xf numFmtId="167" fontId="10" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1927,7 +1938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="42" customWidth="1" style="31" min="1" max="1"/>
@@ -2313,30 +2324,30 @@
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  Hetzner Volume (100GB)</t>
         </is>
       </c>
-      <c r="B32" t="n">
+      <c r="B32" s="31" t="n">
         <v>5.2</v>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="31" t="inlineStr">
         <is>
           <t>Block storage @ €0.052/GB — disk/DB headroom (active)</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="32">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  Hetzner Object Storage (backups)</t>
         </is>
       </c>
-      <c r="B33" t="n">
+      <c r="B33" s="31" t="n">
         <v>5.99</v>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="31" t="inlineStr">
         <is>
           <t>S3 bucket — daily DB backups, 14-day retention</t>
         </is>
@@ -2408,14 +2419,6 @@
           <t xml:space="preserve">  Payment processing blended</t>
         </is>
       </c>
-      <c r="B38" s="58" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="C38" s="34" t="inlineStr">
-        <is>
-          <t>Paystack SA + Stripe intl</t>
-        </is>
-      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="32">
       <c r="A39" s="37" t="inlineStr">
@@ -2466,6 +2469,43 @@
       <c r="C42" s="34" t="inlineStr">
         <is>
           <t>Alert fires when AI spend &gt; this % of income</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="62" t="inlineStr">
+        <is>
+          <t>FAILOVER / STANDBY LANE (added 22 Jul 2026 — reconciles Session 142, 18 Jul)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Scaleway standby cost per Mtok, in (USD)</t>
+        </is>
+      </c>
+      <c r="B45" s="63" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Mistral-Medium 3.5 128B — one-model standby row, David's ruling 18 Jul; retired mistral-small ($0.15/$0.35) + qwen3 lanes. Failover-only (Anthropic outage/ban), not the primary billed lane — verify on Scaleway console before any production flip. CHANGELOG Session 142.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Scaleway standby cost per Mtok, out (USD)</t>
+        </is>
+      </c>
+      <c r="B46" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Same source as above — output-token rate.</t>
         </is>
       </c>
     </row>

</xml_diff>